<commit_message>
Layer 5 complete: signals engine, SKIP fix, duplicate column fix, clickable links
</commit_message>
<xml_diff>
--- a/construtoras_enriched.xlsx
+++ b/construtoras_enriched.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="791">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="789">
   <si>
     <t>Ranking</t>
   </si>
@@ -2341,34 +2341,28 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Direcional (DIRR3), MRV (MRVE3), Cury (CURY3): o que esperar das construtoras no 1T26, segundo o Santander (Seu Dinheiro, 2026-05-05) | O grande teste das incorporadoras: quem aguenta mais um ano de crédito caro no setor? Itaú BBA responde (Seu Dinheiro, 2026-04-23) | Direcional Engenharia registra maior VGV de lançamentos da história, com R$ 1,9 bi no segundo trimestre (Diário do Comércio, 2025-08-12)</t>
-  </si>
-  <si>
-    <t>5 melhores construtoras do Minha Casa, Minha Vida! (MANAUSonline.com, 2026-04-23) | Arapongas anuncia novo residencial com 665 novas moradias na Zona Sul (Tribuna do Norte, 2026-04-30)</t>
+    <t>Direcional Engenharia registra maior VGV de lançamentos da história, com R$ 1,9 bi no segundo trimestre (Diário do Comércio, 2025-08-12) | Direcional Engenharia paga comissões com a Split C (Baguete, 2025-11-07) | Programa de estágio: Direcional Engenharia e Rive Incorporadora abrem vagas (IstoÉ Dinheiro, 2022-05-12)</t>
   </si>
   <si>
     <t>MPD Engenharia lança segunda fase do New Time, em São Paulo (Terra, 2026-04-28)</t>
   </si>
   <si>
-    <t>Insider-Favored Growth Companies To Watch In June 2024 (Simply Wall St.· via Yahoo Finance, 2024-05-06) | Three Growth Companies With High Insider Ownership And Up To 60% Earnings Growth (Simply Wall St.· via Yahoo Finance, 2024-05-06)</t>
-  </si>
-  <si>
-    <t>Lucro da Tenda dobra no 1º tri e supera estimativas (Terra, 2026-05-05) | Tenda: Lucro líquido consolidado atinge R$ 183,4 milhões no primeiro trimestre (O POVO, 2026-05-05)</t>
-  </si>
-  <si>
-    <t>Direcional (DIRR3), MRV (MRVE3), Cury (CURY3): o que esperar das construtoras no 1T26, segundo o Santander (Seu Dinheiro, 2026-05-05) | Por que as construtoras despencaram na bolsa hoje? Entenda (Valor Investe, 2026-04-27) | Desempenho desigual: O que esperar das construtoras no 1T26, segundo o Santander (Money Times, 2026-05-05)</t>
+    <t>Insider-Favored Growth Companies To Watch In June 2024 (Simply Wall St.· via Yahoo Finance, 2024-05-08) | Three Growth Companies With High Insider Ownership And Up To 60% Earnings Growth (Simply Wall St.· via Yahoo Finance, 2024-05-08)</t>
+  </si>
+  <si>
+    <t>Tenda (TEND3): lucro dobra no 1º tri, vai a R$ 183,4 milhões e supera estimativas (InfoMoney, 2026-05-05) | Tenda: Lucro líquido consolidado atinge R$ 183,4 milhões no primeiro trimestre (O POVO, 2026-05-06) | Lucro da Tenda dobra no 1º tri e supera estimativas (Terra, 2026-05-05)</t>
+  </si>
+  <si>
+    <t>Direcional (DIRR3), MRV (MRVE3), Cury (CURY3): o que esperar das construtoras no 1T26, segundo o Santander (Seu Dinheiro, 2026-05-05) | Alta de custos é grande vilã de construtoras na B3 – mas analistas veem oportunidades (InfoMoney, 2026-05-07) | Por que as construtoras despencaram na bolsa hoje? Entenda (Valor Investe, 2026-04-27)</t>
   </si>
   <si>
     <t>Famílias da Vila Gomes precisam de uma resposta (O POVO Mais, 2026-04-26)</t>
   </si>
   <si>
-    <t>5 melhores construtoras do Minha Casa, Minha Vida! (MANAUSonline.com, 2026-04-23)</t>
-  </si>
-  <si>
-    <t>5 melhores construtoras do Minha Casa, Minha Vida! (MANAUSonline.com, 2026-04-23) | Incorporadora antecipa decorado em projeto de alto padrão em Curitiba (g1, 2026-04-28) | Construtora deve devolver valor integral do imóvel se entrega atrasar mais de 180 dias (Consultor Jurídico, 2026-04-23)</t>
-  </si>
-  <si>
-    <t>O grande teste das incorporadoras: quem aguenta mais um ano de crédito caro no setor? Itaú BBA responde (Seu Dinheiro, 2026-04-23)</t>
+    <t>Empar lança loteamento em Praia Grande, impulsionado pelo crescimento de Aracruz (A Gazeta, 2026-04-30)</t>
+  </si>
+  <si>
+    <t>Expansão do MCMV estimula incorporadoras a retomar lançamentos para classe média (Estadão, 2026-04-25) | Marquise Incorporações cria The Dream Brokers para corretores (Diário do Nordeste, 2026-05-06) | Empresário é acusado de golpe milionário em Arapiraca (TribunaHoje.com, 2026-04-25)</t>
   </si>
   <si>
     <t>Ribeirão Preto é a 3ª cidade que mais vende imóveis em SP e se consolida como um dos principais mercados do Estado (A Tribuna Regional, 2026-04-24)</t>
@@ -2377,16 +2371,16 @@
     <t>Brasília Square cria nova centralidade em Araçatuba (g1, 2026-04-29)</t>
   </si>
   <si>
-    <t>Impulsionada por Aracruz, Praia Grande ganha novo loteamento com foco em valorização (A Gazeta, 2026-05-01) | De corretor a 'guru do retrofit': ele mudou o Centro de Porto Alegre ao reformar prédios abandonados (Exame, 2026-04-27) | Artista do MoMa assina obra em prédio de luxo nos Jardins, em São Paulo (Exame, 2026-04-26)</t>
-  </si>
-  <si>
-    <t>Trisa Incorporadora: Natureza e sofisticação no Agreste (Folha PE, 2026-04-22) | PDG, Gafisa, Alphaville: incorporadoras em crise lutam para recuperar confiança de investidores (Estadão, 2026-04-24) | Expansão do MCMV estimula incorporadoras a retomar lançamentos para classe média (Estadão, 2026-04-25)</t>
-  </si>
-  <si>
-    <t>Por que as construtoras despencaram na bolsa hoje? Entenda (Valor Investe, 2026-04-27) | O grande teste das incorporadoras: quem aguenta mais um ano de crédito caro no setor? Itaú BBA responde (Seu Dinheiro, 2026-04-23) | A imobiliária e os danos causados por construtoras (Diário do Comércio, 2026-04-24)</t>
-  </si>
-  <si>
-    <t>Empar lança loteamento em Praia Grande, impulsionado pelo crescimento de Aracruz (A Gazeta, 2026-04-30) | Impulsionada por Aracruz, Praia Grande ganha novo loteamento com foco em valorização (A Gazeta, 2026-05-01) | Housi mira R$ 6 bilhões em lançamentos em nova vertical voltada para saúde (Exame, 2026-04-25)</t>
+    <t>Artista do MoMa assina obra em prédio de luxo nos Jardins, em São Paulo (Exame, 2026-04-26)</t>
+  </si>
+  <si>
+    <t>PDG, Gafisa, Alphaville: incorporadoras em crise lutam para recuperar confiança de investidores (Estadão, 2026-04-24) | Incorporadora boutique: especialização que agrega valor (g1, 2026-05-01) | Incorporadora antecipa decorado em projeto de alto padrão em Curitiba (g1, 2026-04-28)</t>
+  </si>
+  <si>
+    <t>Expansão do MCMV estimula incorporadoras a retomar lançamentos para classe média (Estadão, 2026-04-25) | TCE cobra R$ 16,5 mi por rompimento de reservatório que inundou bairro em Florianópolis (ND Mais, 2026-05-05) | Lago Corumbá IV recebe lançamento do Grupo CPR e reorganiza alto padrão de condomínio no Centro-Oeste (O GLOBO, 2026-05-01)</t>
+  </si>
+  <si>
+    <t>Housi mira R$ 6 bilhões em lançamentos em nova vertical voltada para saúde (Exame, 2026-04-25)</t>
   </si>
 </sst>
 </file>
@@ -3012,7 +3006,7 @@
         <v>774</v>
       </c>
       <c r="AB3" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="4" spans="1:28">
@@ -3098,7 +3092,7 @@
         <v>774</v>
       </c>
       <c r="AB4" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="5" spans="1:28">
@@ -3181,7 +3175,7 @@
         <v>774</v>
       </c>
       <c r="AB5" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="6" spans="1:28">
@@ -3264,7 +3258,7 @@
         <v>774</v>
       </c>
       <c r="AB6" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="7" spans="1:28">
@@ -3430,7 +3424,7 @@
         <v>774</v>
       </c>
       <c r="AB8" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="9" spans="1:28">
@@ -3513,7 +3507,7 @@
         <v>774</v>
       </c>
       <c r="AB9" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="10" spans="1:28">
@@ -4254,7 +4248,7 @@
         <v>774</v>
       </c>
       <c r="AB18" t="s">
-        <v>782</v>
+        <v>774</v>
       </c>
     </row>
     <row r="19" spans="1:28">
@@ -5250,7 +5244,7 @@
         <v>774</v>
       </c>
       <c r="AB30" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="31" spans="1:28">
@@ -5745,7 +5739,7 @@
         <v>774</v>
       </c>
       <c r="AB36" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="37" spans="1:28">
@@ -6077,7 +6071,7 @@
         <v>774</v>
       </c>
       <c r="AB40" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="41" spans="1:28">
@@ -6160,7 +6154,7 @@
         <v>774</v>
       </c>
       <c r="AB41" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
     <row r="42" spans="1:28">
@@ -6243,7 +6237,7 @@
         <v>774</v>
       </c>
       <c r="AB42" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="43" spans="1:28">
@@ -6317,7 +6311,7 @@
         <v>774</v>
       </c>
       <c r="AB43" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
     </row>
     <row r="44" spans="1:28">
@@ -6895,7 +6889,7 @@
         <v>774</v>
       </c>
       <c r="AB50" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
     </row>
     <row r="51" spans="1:28">
@@ -7817,7 +7811,7 @@
         <v>774</v>
       </c>
       <c r="AB61" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
     </row>
   </sheetData>

</xml_diff>